<commit_message>
Add Low Budget Investment Insights project and update previous crypto analysis tasks
</commit_message>
<xml_diff>
--- a/Top 5 Crypto Liquidity Analysis/Top_5_Crypto_Liquidity_Analysis.xlsx
+++ b/Top 5 Crypto Liquidity Analysis/Top_5_Crypto_Liquidity_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\elevence skills\data analytics\Top 5 Crypto Liquidity Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{801D5B40-57AB-402A-B90D-3B53672CAB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00831A5B-A4EE-4A7D-BBD9-DE9FDC03A6A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -679,6 +679,90 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -712,6 +796,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -727,6 +816,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -742,6 +836,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -757,6 +856,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -772,6 +876,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -787,6 +896,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-47C1-409F-901A-DFFD3BB74736}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -1530,8 +1644,8 @@
       <xdr:row>8</xdr:row>
       <xdr:rowOff>160021</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="Price_Category">
@@ -1554,7 +1668,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -1598,15 +1712,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>129540</xdr:colOff>
+      <xdr:colOff>579120</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>72390</xdr:rowOff>
+      <xdr:rowOff>102870</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>144780</xdr:colOff>
+      <xdr:colOff>594360</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>72390</xdr:rowOff>
+      <xdr:rowOff>102870</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2264,7 +2378,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D73D9CC-BF2A-43A0-9262-DA856ABEAF37}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D73D9CC-BF2A-43A0-9262-DA856ABEAF37}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0"/>
@@ -2327,12 +2441,84 @@
   <dataFields count="1">
     <dataField name="Sum of Volume_24h" fld="3" baseField="5" baseItem="2" numFmtId="3"/>
   </dataFields>
-  <chartFormats count="1">
+  <chartFormats count="7">
     <chartFormat chart="2" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="10"/>
           </reference>
         </references>
       </pivotArea>

</xml_diff>